<commit_message>
funcionalidad core terminada, falta testing, falta crud de drive y listXlsx,
</commit_message>
<xml_diff>
--- a/LISTAS/ma/SOPAPA COMUN Y GIGANTE DISMAY.xlsx
+++ b/LISTAS/ma/SOPAPA COMUN Y GIGANTE DISMAY.xlsx
@@ -846,7 +846,7 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="36" t="n">
-        <v>45217</v>
+        <v>45231</v>
       </c>
       <c r="E1" s="3" t="n"/>
     </row>
@@ -956,7 +956,7 @@
       </c>
       <c r="C29" s="25" t="n"/>
       <c r="D29" s="21" t="n">
-        <v>271.635</v>
+        <v>298.5</v>
       </c>
     </row>
     <row r="30" ht="19.5" customHeight="1" s="29">
@@ -972,7 +972,7 @@
       </c>
       <c r="C30" s="25" t="n"/>
       <c r="D30" s="21" t="n">
-        <v>203.40866</v>
+        <v>223.526</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="29">

</xml_diff>